<commit_message>
Update student Excel template for improved data import compatibility
</commit_message>
<xml_diff>
--- a/public/excel/Student-template.xlsx
+++ b/public/excel/Student-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Academics\Capstone\BPS-LMS-Admin\public\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{94F03C93-1AD0-4DB7-96FC-28DD702E09AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0226CB06-0100-4721-9507-ABF8B6B3805D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{ADD765D1-D9C8-48DC-9998-CE173B0BFB7F}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="39">
   <si>
     <t>First data column must be blank.</t>
   </si>
@@ -138,6 +138,21 @@
   </si>
   <si>
     <t>Start entering data below this line</t>
+  </si>
+  <si>
+    <t>Data Import Template</t>
+  </si>
+  <si>
+    <t>Data:</t>
+  </si>
+  <si>
+    <t>Students</t>
+  </si>
+  <si>
+    <t>Notes:</t>
+  </si>
+  <si>
+    <t>Please do not change the template headings.</t>
   </si>
 </sst>
 </file>
@@ -529,7 +544,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E0C710AA-4AD7-4A35-9943-DCF1B939226B}">
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="28.6640625" customWidth="1"/>
@@ -537,167 +552,190 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A10" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A11" t="s">
         <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G8" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B9" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>10</v>
-      </c>
-      <c r="E9" t="s">
-        <v>19</v>
-      </c>
-      <c r="F9" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" t="s">
-        <v>22</v>
-      </c>
-      <c r="I9" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="B10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G10" t="s">
-        <v>26</v>
-      </c>
-      <c r="H10" t="s">
-        <v>26</v>
-      </c>
-      <c r="I10" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" t="s">
-        <v>28</v>
-      </c>
-      <c r="E11" t="s">
-        <v>29</v>
-      </c>
-      <c r="F11" t="s">
-        <v>28</v>
-      </c>
-      <c r="G11" t="s">
-        <v>28</v>
-      </c>
-      <c r="H11" t="s">
-        <v>28</v>
-      </c>
-      <c r="I11" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="H12" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B15" t="s">
+        <v>17</v>
+      </c>
+      <c r="C15" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" t="s">
+        <v>10</v>
+      </c>
+      <c r="E15" t="s">
+        <v>19</v>
+      </c>
+      <c r="F15" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" t="s">
+        <v>21</v>
+      </c>
+      <c r="H15" t="s">
+        <v>22</v>
+      </c>
+      <c r="I15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="B16" t="s">
+        <v>25</v>
+      </c>
+      <c r="C16" t="s">
+        <v>26</v>
+      </c>
+      <c r="D16" t="s">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s">
+        <v>26</v>
+      </c>
+      <c r="F16" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" t="s">
+        <v>26</v>
+      </c>
+      <c r="H16" t="s">
+        <v>26</v>
+      </c>
+      <c r="I16" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A17" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B17" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" t="s">
+        <v>28</v>
+      </c>
+      <c r="D17" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17" t="s">
+        <v>28</v>
+      </c>
+      <c r="G17" t="s">
+        <v>28</v>
+      </c>
+      <c r="H17" t="s">
+        <v>28</v>
+      </c>
+      <c r="I17" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A18" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E18" t="s">
+        <v>31</v>
+      </c>
+      <c r="H18" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A19" s="1" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>